<commit_message>
Excel LTV model updated
</commit_message>
<xml_diff>
--- a/excel/ltv_model.xlsx
+++ b/excel/ltv_model.xlsx
@@ -5,20 +5,20 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sridh\reachmobi-portfolio-analysis\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sridh\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{038EEA2D-72BC-4422-A350-DFD5C6FAE046}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1216DF44-1A36-4AF0-AFCE-CA2EAE120FF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="LTV_Projection" sheetId="4" r:id="rId1"/>
-    <sheet name="Payback_Matrix" sheetId="5" r:id="rId2"/>
-    <sheet name="Recommendations" sheetId="6" r:id="rId3"/>
-    <sheet name="data_ltv" sheetId="1" r:id="rId4"/>
-    <sheet name="data_spend" sheetId="2" r:id="rId5"/>
-    <sheet name="data_arpdau" sheetId="3" r:id="rId6"/>
+    <sheet name="LTV_Projection" sheetId="1" r:id="rId1"/>
+    <sheet name="Payback_Matrix" sheetId="2" r:id="rId2"/>
+    <sheet name="Recommendations" sheetId="3" r:id="rId3"/>
+    <sheet name="data_ltv" sheetId="4" r:id="rId4"/>
+    <sheet name="data_spend" sheetId="5" r:id="rId5"/>
+    <sheet name="data_arpdau" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,30 +37,149 @@
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Senior Analyst</author>
+  </authors>
+  <commentList>
+    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000001000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Helper columns (L-S) are computed downstream of the SQL output (A-J). Power-law fit: LTV(d) = a * d^b, fit through D7/D30/D60/D90 actuals.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="69">
+  <si>
+    <t xml:space="preserve">EXECUTIVE RECOMMENDATIONS </t>
+  </si>
+  <si>
+    <t>Budget reallocation summary</t>
+  </si>
+  <si>
+    <t>Current spend on CUT combos:</t>
+  </si>
+  <si>
+    <t>Current spend on HOLD combos:</t>
+  </si>
+  <si>
+    <t>Current spend on TEST combos:</t>
+  </si>
+  <si>
+    <t>Current spend on SCALE combos:</t>
+  </si>
+  <si>
+    <t>Total UA spend (paid channels):</t>
+  </si>
+  <si>
+    <t>% currently going to CUT decisions:</t>
+  </si>
+  <si>
+    <t>Top 3 actions:</t>
+  </si>
+  <si>
+    <t>Reallocation Impact (if all CUT spend redirected to HOLD/TEST):</t>
+  </si>
+  <si>
+    <t>Avg CAC on CUT combos:</t>
+  </si>
+  <si>
+    <t>Avg CAC on HOLD combos:</t>
+  </si>
+  <si>
+    <t>Implied incremental installs from reallocation:</t>
+  </si>
+  <si>
+    <t>(Negative = HOLD CAC higher than CUT CAC, but HOLD users pay back)</t>
+  </si>
+  <si>
+    <t>LTV PROJECTION &amp; PAYBACK MODEL</t>
+  </si>
+  <si>
+    <t>Select channel-app:</t>
+  </si>
+  <si>
+    <t>tiktok_launchpad</t>
+  </si>
+  <si>
+    <t>Cohort size:</t>
+  </si>
+  <si>
+    <t>CAC (true):</t>
+  </si>
+  <si>
+    <t>Day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Actual LTV </t>
+  </si>
+  <si>
+    <t>Projected LTV</t>
+  </si>
+  <si>
+    <t>b (slope):</t>
+  </si>
+  <si>
+    <t>a (intercept):</t>
+  </si>
+  <si>
+    <t>Payback day:</t>
+  </si>
+  <si>
+    <t>ROAS at D365:</t>
+  </si>
+  <si>
+    <t>ROAS at D540:</t>
+  </si>
+  <si>
+    <t>Verdict:</t>
+  </si>
+  <si>
+    <t>PAYBACK MATRIX — Projected Payback Day by Channel × App</t>
+  </si>
+  <si>
+    <t>Channel ↓ / App →</t>
+  </si>
+  <si>
+    <t>inboxzen</t>
+  </si>
+  <si>
+    <t>launchpad</t>
+  </si>
+  <si>
+    <t>pingme</t>
+  </si>
+  <si>
+    <t>wallcraft</t>
+  </si>
+  <si>
+    <t>applovin</t>
+  </si>
+  <si>
+    <t>google</t>
+  </si>
+  <si>
+    <t>meta</t>
+  </si>
+  <si>
+    <t>tiktok</t>
+  </si>
+  <si>
+    <t>VERDICT MATRIX</t>
+  </si>
   <si>
     <t>channel</t>
   </si>
@@ -92,36 +211,33 @@
     <t>payback_bucket</t>
   </si>
   <si>
-    <t>tiktok</t>
-  </si>
-  <si>
-    <t>inboxzen</t>
+    <t>combo_key</t>
+  </si>
+  <si>
+    <t>b_slope</t>
+  </si>
+  <si>
+    <t>a_intercept</t>
+  </si>
+  <si>
+    <t>proj_ltv_d180</t>
+  </si>
+  <si>
+    <t>proj_ltv_d365</t>
+  </si>
+  <si>
+    <t>payback_day</t>
+  </si>
+  <si>
+    <t>verdict</t>
+  </si>
+  <si>
+    <t>total_spend</t>
   </si>
   <si>
     <t>unprofitable at D90</t>
   </si>
   <si>
-    <t>applovin</t>
-  </si>
-  <si>
-    <t>launchpad</t>
-  </si>
-  <si>
-    <t>meta</t>
-  </si>
-  <si>
-    <t>google</t>
-  </si>
-  <si>
-    <t>wallcraft</t>
-  </si>
-  <si>
-    <t>pingme</t>
-  </si>
-  <si>
-    <t>total_spend</t>
-  </si>
-  <si>
     <t>true_installs</t>
   </si>
   <si>
@@ -146,123 +262,25 @@
     <t>arpdau_total</t>
   </si>
   <si>
-    <t>combo_key</t>
-  </si>
-  <si>
-    <t>b_slope</t>
-  </si>
-  <si>
-    <t>a_intercept</t>
-  </si>
-  <si>
-    <t>proj_ltv_d180</t>
-  </si>
-  <si>
-    <t>proj_ltv_d365</t>
-  </si>
-  <si>
-    <t>payback_day</t>
-  </si>
-  <si>
-    <t>verdict</t>
-  </si>
-  <si>
-    <t>LTV PROJECTION &amp; PAYBACK MODEL</t>
-  </si>
-  <si>
-    <t>Select channel-app:</t>
-  </si>
-  <si>
-    <t>Cohort size:</t>
-  </si>
-  <si>
-    <t>CAC (true):</t>
-  </si>
-  <si>
-    <t>Day</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Actual LTV </t>
-  </si>
-  <si>
-    <t>Projected LTV</t>
-  </si>
-  <si>
-    <t>b (slope):</t>
-  </si>
-  <si>
-    <t>a (intercept):</t>
-  </si>
-  <si>
-    <t>Payback day:</t>
-  </si>
-  <si>
-    <t>ROAS at D365:</t>
-  </si>
-  <si>
-    <t>ROAS at D540:</t>
-  </si>
-  <si>
-    <t>Verdict:</t>
-  </si>
-  <si>
-    <t>tiktok_launchpad</t>
-  </si>
-  <si>
-    <t>PAYBACK MATRIX — Projected Payback Day by Channel × App</t>
-  </si>
-  <si>
-    <t>Channel ↓ / App →</t>
-  </si>
-  <si>
-    <t>VERDICT MATRIX</t>
-  </si>
-  <si>
-    <r>
-      <t>EXECUTIVE RECOMMENDATIONS</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
-    <t>Budget reallocation summary</t>
-  </si>
-  <si>
-    <t>Current spend on CUT combos:</t>
-  </si>
-  <si>
-    <t>Current spend on HOLD combos:</t>
-  </si>
-  <si>
-    <t>Current spend on TEST combos:</t>
-  </si>
-  <si>
-    <t>Current spend on SCALE combos:</t>
-  </si>
-  <si>
-    <t>Total UA spend (paid channels):</t>
-  </si>
-  <si>
-    <t>% currently going to CUT decisions:</t>
-  </si>
-  <si>
-    <t>Top 3 actions:</t>
+    <t>1. Cut all PingMe paid acquisition immediately (~$49K/period across 4 channels, 15% of UA budget). All paid PingMe combos project &gt;665-day payback. PingMe's $0.05 ARPDAU cannot support any meaningful CAC.It's best to keep organic only.</t>
+  </si>
+  <si>
+    <t>2. Reallocate Meta + Google launchpad + wallcraft spend (~$107K) to better performing channels. Meta_launchpad payback is 377 days (CUT) while tiktok_launchpad is 264 days (HOLD). same app, but better economics.</t>
+  </si>
+  <si>
+    <t>3. Cautiously TEST tiktok_inboxzen and applovin_inboxzen (~$19.5K combined) with a strict D180 ROAS &gt;= 1.0 gate. These are the only combos projecting sub-180-day payback.It's good to monitor weekly.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
+  </numFmts>
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -303,11 +321,27 @@
     </font>
     <font>
       <b/>
-      <sz val="14"/>
-      <color theme="1"/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -354,23 +388,74 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF8696B"/>
+          <bgColor rgb="FFF8696B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB84"/>
+          <bgColor rgb="FFFFEB84"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF63BE7B"/>
+          <bgColor rgb="FF63BE7B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -387,15 +472,8 @@
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
+  <c:roundedCorners val="1"/>
+  <c:style val="2"/>
   <c:chart>
     <c:title>
       <c:tx>
@@ -404,7 +482,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:defRPr sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -417,7 +495,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
+              <a:rPr lang="en-US" sz="1400" b="0" i="0" strike="noStrike" baseline="0"/>
               <a:t>LTV Curve: Actual (D7–D90) and Power-Law Projection (D180–D540)</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
@@ -428,7 +506,7 @@
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.18221234180018642"/>
+          <c:x val="0.18221234180018639"/>
           <c:y val="4.0243140282359452E-2"/>
         </c:manualLayout>
       </c:layout>
@@ -437,29 +515,9 @@
         <a:noFill/>
         <a:ln>
           <a:noFill/>
+          <a:prstDash val="solid"/>
         </a:ln>
-        <a:effectLst/>
       </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
@@ -468,7 +526,7 @@
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
-          <c:idx val="1"/>
+          <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
             <c:v>Actual</c:v>
@@ -478,9 +536,9 @@
               <a:solidFill>
                 <a:schemeClr val="accent2"/>
               </a:solidFill>
+              <a:prstDash val="solid"/>
               <a:round/>
             </a:ln>
-            <a:effectLst/>
           </c:spPr>
           <c:marker>
             <c:symbol val="none"/>
@@ -530,12 +588,12 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-5C60-4FBD-AD3D-84A6253D8ADD}"/>
+              <c16:uniqueId val="{00000000-740D-4651-8DC9-E8CF7EDDF22B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="0"/>
+          <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
             <c:v>Projected</c:v>
@@ -545,9 +603,9 @@
               <a:solidFill>
                 <a:schemeClr val="accent1"/>
               </a:solidFill>
+              <a:prstDash val="solid"/>
               <a:round/>
             </a:ln>
-            <a:effectLst/>
           </c:spPr>
           <c:marker>
             <c:symbol val="none"/>
@@ -615,7 +673,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-5C60-4FBD-AD3D-84A6253D8ADD}"/>
+              <c16:uniqueId val="{00000001-740D-4651-8DC9-E8CF7EDDF22B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -644,7 +702,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -673,29 +731,9 @@
             <a:noFill/>
             <a:ln>
               <a:noFill/>
+              <a:prstDash val="solid"/>
             </a:ln>
-            <a:effectLst/>
           </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
@@ -710,16 +748,16 @@
                 <a:lumOff val="85000"/>
               </a:schemeClr>
             </a:solidFill>
+            <a:prstDash val="solid"/>
             <a:round/>
           </a:ln>
-          <a:effectLst/>
         </c:spPr>
         <c:txPr>
           <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -754,9 +792,9 @@
                   <a:lumOff val="85000"/>
                 </a:schemeClr>
               </a:solidFill>
+              <a:prstDash val="solid"/>
               <a:round/>
             </a:ln>
-            <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
         <c:title>
@@ -766,7 +804,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -795,29 +833,9 @@
             <a:noFill/>
             <a:ln>
               <a:noFill/>
+              <a:prstDash val="solid"/>
             </a:ln>
-            <a:effectLst/>
           </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
@@ -827,15 +845,15 @@
           <a:noFill/>
           <a:ln>
             <a:noFill/>
+            <a:prstDash val="solid"/>
           </a:ln>
-          <a:effectLst/>
         </c:spPr>
         <c:txPr>
           <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -854,13 +872,6 @@
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
@@ -869,15 +880,15 @@
         <a:noFill/>
         <a:ln>
           <a:noFill/>
+          <a:prstDash val="solid"/>
         </a:ln>
-        <a:effectLst/>
       </c:spPr>
       <c:txPr>
         <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+            <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -895,14 +906,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
+    <c:showDLblsOverMax val="1"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -915,569 +919,16 @@
           <a:lumOff val="85000"/>
         </a:schemeClr>
       </a:solidFill>
+      <a:prstDash val="solid"/>
       <a:round/>
     </a:ln>
-    <a:effectLst/>
   </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
   <c:printSettings>
     <c:headerFooter/>
     <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
-</file>
-
-<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="332">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1497,10 +948,10 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Chart 2">
+        <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F8031EB4-F4D0-9991-373B-FA425D9D8DE0}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1805,7 +1256,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA035669-38F0-4E59-8EC9-8441C3397A32}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
@@ -1814,22 +1265,22 @@
     <col min="5" max="5" width="14.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18">
+    <row r="1" spans="1:5" ht="18" customHeight="1">
       <c r="A1" s="6" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="3" t="s">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>48</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="3" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="B5" s="3">
         <f>INDEX(data_ltv!C:C, MATCH(B3, data_ltv!L:L, 0))</f>
@@ -1838,7 +1289,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="3" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="B6">
         <f>INDEX(data_ltv!D:D, MATCH(B3, data_ltv!L:L, 0))</f>
@@ -1847,16 +1298,16 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="3" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="D8" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="E8" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1871,7 +1322,7 @@
         <v>7</v>
       </c>
       <c r="E9">
-        <f>$B$18*D9^$B$17</f>
+        <f t="shared" ref="E9:E15" si="0">$B$18*D9^$B$17</f>
         <v>0.15930214456482322</v>
       </c>
     </row>
@@ -1887,7 +1338,7 @@
         <v>30</v>
       </c>
       <c r="E10">
-        <f t="shared" ref="E10:E15" si="0">$B$18*D10^$B$17</f>
+        <f t="shared" si="0"/>
         <v>0.44381174463369893</v>
       </c>
     </row>
@@ -1952,25 +1403,25 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B17" s="3" cm="1">
+        <v>22</v>
+      </c>
+      <c r="B17" s="3">
         <f t="array" ref="B17">SLOPE(LN(B9:B12), LN(A9:A12))</f>
         <v>0.7040519367834055</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B18" s="3" cm="1">
+        <v>23</v>
+      </c>
+      <c r="B18" s="3">
         <f t="array" ref="B18">EXP(INTERCEPT(LN(B9:B12), LN(A9:A12)))</f>
         <v>4.0478900781559579E-2</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="3" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="B20" s="3">
         <f>IF(B17&gt;0, (B6/B18)^(1/B17), "N/A")</f>
@@ -1979,7 +1430,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="B21" s="3">
         <f>E14/B6</f>
@@ -1988,7 +1439,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="3" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="B22" s="3">
         <f>E15/B6</f>
@@ -1997,7 +1448,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="B23" s="3" t="str">
         <f>IF(ISNUMBER(B20), IF(B20&lt;=90,"SCALE",IF(B20&lt;=180,"TEST",IF(B20&lt;=365,"HOLD","CUT"))), "CUT")</f>
@@ -2007,23 +1458,11 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{31B7F4CF-DABF-4C8F-BF9E-F015D5D6F519}">
-          <x14:formula1>
-            <xm:f>data_ltv!$L$2:$L$17</xm:f>
-          </x14:formula1>
-          <xm:sqref>B3</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A666FC8-2875-42C5-97AD-EBD8F7694F50}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
@@ -2032,247 +1471,241 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>49</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="3" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4">
+        <v>34</v>
+      </c>
+      <c r="B4" s="7">
         <f>INDEX(data_ltv!Q:Q, MATCH($A4&amp;"_"&amp;B$3, data_ltv!L:L, 0))</f>
         <v>171.97383024385215</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="7">
         <f>INDEX(data_ltv!Q:Q, MATCH($A4&amp;"_"&amp;C$3, data_ltv!L:L, 0))</f>
         <v>705.89068398840459</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="7">
         <f>INDEX(data_ltv!Q:Q, MATCH($A4&amp;"_"&amp;D$3, data_ltv!L:L, 0))</f>
         <v>664.73093422199565</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="7">
         <f>INDEX(data_ltv!Q:Q,MATCH($A4&amp;"_"&amp;E$3,data_ltv!L:L,0))</f>
         <v>2244.4036168319763</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5">
+        <v>35</v>
+      </c>
+      <c r="B5" s="7">
         <f>INDEX(data_ltv!Q:Q, MATCH($A5&amp;"_"&amp;B$3, data_ltv!L:L, 0))</f>
         <v>228.72583990645708</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="7">
         <f>INDEX(data_ltv!Q:Q, MATCH($A5&amp;"_"&amp;C$3, data_ltv!L:L, 0))</f>
         <v>329.61801468014573</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="7">
         <f>INDEX(data_ltv!Q:Q, MATCH($A5&amp;"_"&amp;D$3, data_ltv!L:L, 0))</f>
         <v>867.69954894135617</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="7">
         <f>INDEX(data_ltv!Q:Q,MATCH($A5&amp;"_"&amp;E$3,data_ltv!L:L,0))</f>
         <v>402.03673591550307</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6">
+        <v>36</v>
+      </c>
+      <c r="B6" s="7">
         <f>INDEX(data_ltv!Q:Q, MATCH($A6&amp;"_"&amp;B$3, data_ltv!L:L, 0))</f>
         <v>220.01767046274145</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="7">
         <f>INDEX(data_ltv!Q:Q, MATCH($A6&amp;"_"&amp;C$3, data_ltv!L:L, 0))</f>
         <v>377.28086975260862</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="7">
         <f>INDEX(data_ltv!Q:Q, MATCH($A6&amp;"_"&amp;D$3, data_ltv!L:L, 0))</f>
         <v>1140.460728670274</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="7">
         <f>INDEX(data_ltv!Q:Q,MATCH($A6&amp;"_"&amp;E$3,data_ltv!L:L,0))</f>
         <v>449.90250720317772</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
+        <v>37</v>
+      </c>
+      <c r="B7" s="7">
         <f>INDEX(data_ltv!Q:Q, MATCH($A7&amp;"_"&amp;B$3, data_ltv!L:L, 0))</f>
         <v>162.48764019732181</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="7">
         <f>INDEX(data_ltv!Q:Q, MATCH($A7&amp;"_"&amp;C$3, data_ltv!L:L, 0))</f>
         <v>263.64642682689936</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="7">
         <f>INDEX(data_ltv!Q:Q, MATCH($A7&amp;"_"&amp;D$3, data_ltv!L:L, 0))</f>
         <v>749.26972565236929</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="7">
         <f>INDEX(data_ltv!Q:Q,MATCH($A7&amp;"_"&amp;E$3,data_ltv!L:L,0))</f>
         <v>451.7257517761297</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="3" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="D11" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" t="str">
+        <v>34</v>
+      </c>
+      <c r="B12" s="8" t="str">
         <f>INDEX(data_ltv!R:R, MATCH($A12&amp;"_"&amp;B$11, data_ltv!L:L, 0))</f>
         <v>TEST</v>
       </c>
-      <c r="C12" t="str">
+      <c r="C12" s="8" t="str">
         <f>INDEX(data_ltv!R:R, MATCH($A12&amp;"_"&amp;C$11, data_ltv!L:L, 0))</f>
         <v>CUT</v>
       </c>
-      <c r="D12" t="str">
+      <c r="D12" s="8" t="str">
         <f>INDEX(data_ltv!R:R, MATCH($A12&amp;"_"&amp;D$11, data_ltv!L:L, 0))</f>
         <v>CUT</v>
       </c>
-      <c r="E12" t="str">
+      <c r="E12" s="8" t="str">
         <f>INDEX(data_ltv!R:R, MATCH($A12&amp;"_"&amp;E$11, data_ltv!L:L, 0))</f>
         <v>CUT</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" t="str">
+        <v>35</v>
+      </c>
+      <c r="B13" s="8" t="str">
         <f>INDEX(data_ltv!R:R, MATCH($A13&amp;"_"&amp;B$11, data_ltv!L:L, 0))</f>
         <v>HOLD</v>
       </c>
-      <c r="C13" t="str">
+      <c r="C13" s="8" t="str">
         <f>INDEX(data_ltv!R:R, MATCH($A13&amp;"_"&amp;C$11, data_ltv!L:L, 0))</f>
         <v>HOLD</v>
       </c>
-      <c r="D13" t="str">
+      <c r="D13" s="8" t="str">
         <f>INDEX(data_ltv!R:R, MATCH($A13&amp;"_"&amp;D$11, data_ltv!L:L, 0))</f>
         <v>CUT</v>
       </c>
-      <c r="E13" t="str">
+      <c r="E13" s="8" t="str">
         <f>INDEX(data_ltv!R:R, MATCH($A13&amp;"_"&amp;E$11, data_ltv!L:L, 0))</f>
         <v>CUT</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" t="str">
+        <v>36</v>
+      </c>
+      <c r="B14" s="8" t="str">
         <f>INDEX(data_ltv!R:R, MATCH($A14&amp;"_"&amp;B$11, data_ltv!L:L, 0))</f>
         <v>HOLD</v>
       </c>
-      <c r="C14" t="str">
+      <c r="C14" s="8" t="str">
         <f>INDEX(data_ltv!R:R, MATCH($A14&amp;"_"&amp;C$11, data_ltv!L:L, 0))</f>
         <v>CUT</v>
       </c>
-      <c r="D14" t="str">
+      <c r="D14" s="8" t="str">
         <f>INDEX(data_ltv!R:R, MATCH($A14&amp;"_"&amp;D$11, data_ltv!L:L, 0))</f>
         <v>CUT</v>
       </c>
-      <c r="E14" t="str">
+      <c r="E14" s="8" t="str">
         <f>INDEX(data_ltv!R:R, MATCH($A14&amp;"_"&amp;E$11, data_ltv!L:L, 0))</f>
         <v>CUT</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B15" t="str">
+        <v>37</v>
+      </c>
+      <c r="B15" s="8" t="str">
         <f>INDEX(data_ltv!R:R, MATCH($A15&amp;"_"&amp;B$11, data_ltv!L:L, 0))</f>
         <v>TEST</v>
       </c>
-      <c r="C15" t="str">
+      <c r="C15" s="8" t="str">
         <f>INDEX(data_ltv!R:R, MATCH($A15&amp;"_"&amp;C$11, data_ltv!L:L, 0))</f>
         <v>HOLD</v>
       </c>
-      <c r="D15" t="str">
+      <c r="D15" s="8" t="str">
         <f>INDEX(data_ltv!R:R, MATCH($A15&amp;"_"&amp;D$11, data_ltv!L:L, 0))</f>
         <v>CUT</v>
       </c>
-      <c r="E15" t="str">
+      <c r="E15" s="8" t="str">
         <f>INDEX(data_ltv!R:R, MATCH($A15&amp;"_"&amp;E$11, data_ltv!L:L, 0))</f>
         <v>CUT</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B4:B7">
-    <cfRule type="colorScale" priority="3">
+  <conditionalFormatting sqref="B4:E7">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
+        <cfvo type="num" val="90"/>
+        <cfvo type="num" val="200"/>
+        <cfvo type="num" val="540"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
         <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:E15">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFFEF9C"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
+      <formula>"SCALE"</formula>
     </cfRule>
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+      <formula>"TEST"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="4" operator="equal">
+      <formula>"HOLD"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="5" operator="equal">
+      <formula>"CUT"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2280,80 +1713,133 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B0C39DB-2723-4BD2-84B6-9D96DCE2039E}">
-  <dimension ref="A1:B11"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="45.36328125" customWidth="1"/>
+    <col min="1" max="1" width="110" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.5">
-      <c r="A1" s="6" t="s">
-        <v>52</v>
+    <row r="1" spans="1:2" ht="18.5" customHeight="1">
+      <c r="A1" s="9" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="5" t="s">
-        <v>53</v>
+      <c r="A3" s="10" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="11">
         <f>SUMIFS(data_ltv!S:S, data_ltv!R:R, "CUT")</f>
         <v>187378.22999999998</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="B5" s="11">
         <f>SUMIFS(data_ltv!S:S, data_ltv!R:R, "HOLD")</f>
         <v>123201.70000000001</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="B6" s="11">
         <f>SUMIFS(data_ltv!S:S, data_ltv!R:R, "TEST")</f>
         <v>19551.62</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>57</v>
-      </c>
-      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="B7" s="11">
         <f>SUMIFS(data_ltv!S:S, data_ltv!R:R, "SCALE")</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>58</v>
-      </c>
-      <c r="B8">
+        <v>6</v>
+      </c>
+      <c r="B8" s="11">
         <f>SUM(B4:B7)</f>
         <v>330131.55</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="B9" s="3">
+        <v>7</v>
+      </c>
+      <c r="B9" s="12">
         <f>B4/B8</f>
         <v>0.56758655754047138</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
-      <c r="A11" s="3" t="s">
-        <v>60</v>
+    <row r="11" spans="1:2" ht="15.5">
+      <c r="A11" s="13" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="60" customHeight="1">
+      <c r="A12" s="14" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="60" customHeight="1">
+      <c r="A13" s="14" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="60" customHeight="1">
+      <c r="A14" s="14" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17" s="15">
+        <f>SUMPRODUCT(data_ltv!D2:D17, data_ltv!C2:C17, (data_ltv!R2:R17="CUT")*1) / SUMPRODUCT(data_ltv!C2:C17, (data_ltv!R2:R17="CUT")*1)</f>
+        <v>2.8092243274994733</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18" s="15">
+        <f>SUMPRODUCT(data_ltv!D2:D17, data_ltv!C2:C17, (data_ltv!R2:R17="HOLD")*1) / SUMPRODUCT(data_ltv!C2:C17, (data_ltv!R2:R17="HOLD")*1)</f>
+        <v>2.9008722579425115</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="16">
+        <f>B4/B18 - B4/B17</f>
+        <v>-2107.3019505126504</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="17" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -2362,7 +1848,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:S17"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
@@ -2376,66 +1862,66 @@
   <sheetData>
     <row r="1" spans="1:19">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>41</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>42</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>44</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>30</v>
+        <v>51</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>19</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:19">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="C2">
         <v>3479</v>
@@ -2459,34 +1945,34 @@
         <v>0.56999999999999995</v>
       </c>
       <c r="J2" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="L2" t="str">
-        <f>A2&amp;"_"&amp;B2</f>
+        <f t="shared" ref="L2:L17" si="0">A2&amp;"_"&amp;B2</f>
         <v>tiktok_inboxzen</v>
       </c>
-      <c r="M2" cm="1">
+      <c r="M2">
         <f t="array" ref="M2">SLOPE(LN(E2:H2),LN({7,30,60,90}))</f>
         <v>0.90339200746709947</v>
       </c>
-      <c r="N2" cm="1">
+      <c r="N2">
         <f t="array" ref="N2">EXP(INTERCEPT(LN(E2:H2), LN({7,30,60,90})))</f>
         <v>2.1033370343505629E-2</v>
       </c>
       <c r="O2">
-        <f>N2*180^M2</f>
+        <f t="shared" ref="O2:O17" si="1">N2*180^M2</f>
         <v>2.2924719183279767</v>
       </c>
       <c r="P2">
-        <f>N2*365^M2</f>
+        <f t="shared" ref="P2:P17" si="2">N2*365^M2</f>
         <v>4.3417395057821437</v>
       </c>
-      <c r="Q2" s="3">
-        <f>IF(M2&gt;0, (D2/N2)^(1/M2), 9999)</f>
+      <c r="Q2" s="18">
+        <f t="shared" ref="Q2:Q17" si="3">IF(M2&gt;0, (D2/N2)^(1/M2), 9999)</f>
         <v>162.48764019732181</v>
       </c>
       <c r="R2" t="str">
-        <f>IF(Q2&lt;=90,"SCALE",IF(Q2&lt;=180,"TEST",IF(Q2&lt;=365,"HOLD","CUT")))</f>
+        <f t="shared" ref="R2:R17" si="4">IF(Q2&lt;=90,"SCALE",IF(Q2&lt;=180,"TEST",IF(Q2&lt;=365,"HOLD","CUT")))</f>
         <v>TEST</v>
       </c>
       <c r="S2">
@@ -2496,10 +1982,10 @@
     </row>
     <row r="3" spans="1:19">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="C3">
         <v>1363</v>
@@ -2523,34 +2009,34 @@
         <v>0.52</v>
       </c>
       <c r="J3" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="L3" t="str">
-        <f t="shared" ref="L3:L17" si="0">A3&amp;"_"&amp;B3</f>
+        <f t="shared" si="0"/>
         <v>applovin_inboxzen</v>
       </c>
-      <c r="M3" cm="1">
+      <c r="M3">
         <f t="array" ref="M3">SLOPE(LN(E3:H3), LN({7,30,60,90}))</f>
         <v>0.92652162752113265</v>
       </c>
-      <c r="N3" cm="1">
+      <c r="N3">
         <f t="array" ref="N3">EXP(INTERCEPT(LN(E3:H3), LN({7,30,60,90})))</f>
         <v>1.527806232224584E-2</v>
       </c>
       <c r="O3">
-        <f t="shared" ref="O3:O17" si="1">N3*180^M3</f>
+        <f t="shared" si="1"/>
         <v>1.8777035579835606</v>
       </c>
       <c r="P3">
-        <f t="shared" ref="P3:P17" si="2">N3*365^M3</f>
+        <f t="shared" si="2"/>
         <v>3.6148312845913662</v>
       </c>
-      <c r="Q3" s="3">
-        <f t="shared" ref="Q3:Q17" si="3">IF(M3&gt;0, (D3/N3)^(1/M3), 9999)</f>
+      <c r="Q3" s="18">
+        <f t="shared" si="3"/>
         <v>171.97383024385215</v>
       </c>
       <c r="R3" t="str">
-        <f t="shared" ref="R3:R17" si="4">IF(Q3&lt;=90,"SCALE",IF(Q3&lt;=180,"TEST",IF(Q3&lt;=365,"HOLD","CUT")))</f>
+        <f t="shared" si="4"/>
         <v>TEST</v>
       </c>
       <c r="S3">
@@ -2560,10 +2046,10 @@
     </row>
     <row r="4" spans="1:19">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="C4">
         <v>7890</v>
@@ -2587,17 +2073,17 @@
         <v>0.47</v>
       </c>
       <c r="J4" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="L4" t="str">
         <f t="shared" si="0"/>
         <v>tiktok_launchpad</v>
       </c>
-      <c r="M4" cm="1">
+      <c r="M4">
         <f t="array" ref="M4">SLOPE(LN(E4:H4), LN({7,30,60,90}))</f>
         <v>0.7040519367834055</v>
       </c>
-      <c r="N4" cm="1">
+      <c r="N4">
         <f t="array" ref="N4">EXP(INTERCEPT(LN(E4:H4), LN({7,30,60,90})))</f>
         <v>4.0478900781559579E-2</v>
       </c>
@@ -2609,7 +2095,7 @@
         <f t="shared" si="2"/>
         <v>2.5776026193458392</v>
       </c>
-      <c r="Q4" s="3">
+      <c r="Q4" s="18">
         <f t="shared" si="3"/>
         <v>263.64642682689936</v>
       </c>
@@ -2624,10 +2110,10 @@
     </row>
     <row r="5" spans="1:19">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="C5">
         <v>4175</v>
@@ -2651,17 +2137,17 @@
         <v>0.44</v>
       </c>
       <c r="J5" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="L5" t="str">
         <f t="shared" si="0"/>
         <v>meta_inboxzen</v>
       </c>
-      <c r="M5" cm="1">
+      <c r="M5">
         <f t="array" ref="M5">SLOPE(LN(E5:H5), LN({7,30,60,90}))</f>
         <v>0.88312321977618025</v>
       </c>
-      <c r="N5" cm="1">
+      <c r="N5">
         <f t="array" ref="N5">EXP(INTERCEPT(LN(E5:H5), LN({7,30,60,90})))</f>
         <v>2.731940987297328E-2</v>
       </c>
@@ -2673,7 +2159,7 @@
         <f t="shared" si="2"/>
         <v>5.0037043202603204</v>
       </c>
-      <c r="Q5" s="3">
+      <c r="Q5" s="18">
         <f t="shared" si="3"/>
         <v>220.01767046274145</v>
       </c>
@@ -2688,10 +2174,10 @@
     </row>
     <row r="6" spans="1:19">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="C6">
         <v>2778</v>
@@ -2715,17 +2201,17 @@
         <v>0.43</v>
       </c>
       <c r="J6" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="L6" t="str">
         <f t="shared" si="0"/>
         <v>google_inboxzen</v>
       </c>
-      <c r="M6" cm="1">
+      <c r="M6">
         <f t="array" ref="M6">SLOPE(LN(E6:H6), LN({7,30,60,90}))</f>
         <v>0.88251738688269199</v>
       </c>
-      <c r="N6" cm="1">
+      <c r="N6">
         <f t="array" ref="N6">EXP(INTERCEPT(LN(E6:H6), LN({7,30,60,90})))</f>
         <v>2.9217159595933059E-2</v>
       </c>
@@ -2737,7 +2223,7 @@
         <f t="shared" si="2"/>
         <v>5.3321946648884087</v>
       </c>
-      <c r="Q6" s="3">
+      <c r="Q6" s="18">
         <f t="shared" si="3"/>
         <v>228.72583990645708</v>
       </c>
@@ -2752,10 +2238,10 @@
     </row>
     <row r="7" spans="1:19">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="C7">
         <v>6309</v>
@@ -2779,17 +2265,17 @@
         <v>0.4</v>
       </c>
       <c r="J7" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="L7" t="str">
         <f t="shared" si="0"/>
         <v>google_launchpad</v>
       </c>
-      <c r="M7" cm="1">
+      <c r="M7">
         <f t="array" ref="M7">SLOPE(LN(E7:H7), LN({7,30,60,90}))</f>
         <v>0.70791037382651834</v>
       </c>
-      <c r="N7" cm="1">
+      <c r="N7">
         <f t="array" ref="N7">EXP(INTERCEPT(LN(E7:H7), LN({7,30,60,90})))</f>
         <v>5.7583672808929648E-2</v>
       </c>
@@ -2801,7 +2287,7 @@
         <f t="shared" si="2"/>
         <v>3.7512245429776376</v>
       </c>
-      <c r="Q7" s="3">
+      <c r="Q7" s="18">
         <f t="shared" si="3"/>
         <v>329.61801468014573</v>
       </c>
@@ -2816,10 +2302,10 @@
     </row>
     <row r="8" spans="1:19">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="C8">
         <v>3479</v>
@@ -2843,17 +2329,17 @@
         <v>0.39</v>
       </c>
       <c r="J8" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="L8" t="str">
         <f t="shared" si="0"/>
         <v>tiktok_wallcraft</v>
       </c>
-      <c r="M8" cm="1">
+      <c r="M8">
         <f t="array" ref="M8">SLOPE(LN(E8:H8), LN({7,30,60,90}))</f>
         <v>0.59296718879736865</v>
       </c>
-      <c r="N8" cm="1">
+      <c r="N8">
         <f t="array" ref="N8">EXP(INTERCEPT(LN(E8:H8), LN({7,30,60,90})))</f>
         <v>5.6504389233365426E-2</v>
       </c>
@@ -2865,7 +2351,7 @@
         <f t="shared" si="2"/>
         <v>1.868262005072612</v>
       </c>
-      <c r="Q8" s="3">
+      <c r="Q8" s="18">
         <f t="shared" si="3"/>
         <v>451.7257517761297</v>
       </c>
@@ -2880,10 +2366,10 @@
     </row>
     <row r="9" spans="1:19">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="C9">
         <v>2778</v>
@@ -2907,17 +2393,17 @@
         <v>0.39</v>
       </c>
       <c r="J9" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="L9" t="str">
         <f t="shared" si="0"/>
         <v>google_wallcraft</v>
       </c>
-      <c r="M9" cm="1">
+      <c r="M9">
         <f t="array" ref="M9">SLOPE(LN(E9:H9), LN({7,30,60,90}))</f>
         <v>0.63574560276317937</v>
       </c>
-      <c r="N9" cm="1">
+      <c r="N9">
         <f t="array" ref="N9">EXP(INTERCEPT(LN(E9:H9), LN({7,30,60,90})))</f>
         <v>7.7563361907928202E-2</v>
       </c>
@@ -2929,7 +2415,7 @@
         <f t="shared" si="2"/>
         <v>3.3008291538217809</v>
       </c>
-      <c r="Q9" s="3">
+      <c r="Q9" s="18">
         <f t="shared" si="3"/>
         <v>402.03673591550307</v>
       </c>
@@ -2944,10 +2430,10 @@
     </row>
     <row r="10" spans="1:19">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="C10">
         <v>9471</v>
@@ -2971,17 +2457,17 @@
         <v>0.37</v>
       </c>
       <c r="J10" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="L10" t="str">
         <f t="shared" si="0"/>
         <v>meta_launchpad</v>
       </c>
-      <c r="M10" cm="1">
+      <c r="M10">
         <f t="array" ref="M10">SLOPE(LN(E10:H10), LN({7,30,60,90}))</f>
         <v>0.69353902506528642</v>
       </c>
-      <c r="N10" cm="1">
+      <c r="N10">
         <f t="array" ref="N10">EXP(INTERCEPT(LN(E10:H10), LN({7,30,60,90})))</f>
         <v>5.1602352363589385E-2</v>
       </c>
@@ -2993,7 +2479,7 @@
         <f t="shared" si="2"/>
         <v>3.0883008084983987</v>
       </c>
-      <c r="Q10" s="3">
+      <c r="Q10" s="18">
         <f t="shared" si="3"/>
         <v>377.28086975260862</v>
       </c>
@@ -3008,10 +2494,10 @@
     </row>
     <row r="11" spans="1:19">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="C11">
         <v>4175</v>
@@ -3035,17 +2521,17 @@
         <v>0.37</v>
       </c>
       <c r="J11" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="L11" t="str">
         <f t="shared" si="0"/>
         <v>meta_wallcraft</v>
       </c>
-      <c r="M11" cm="1">
+      <c r="M11">
         <f t="array" ref="M11">SLOPE(LN(E11:H11), LN({7,30,60,90}))</f>
         <v>0.62755718500799473</v>
       </c>
-      <c r="N11" cm="1">
+      <c r="N11">
         <f t="array" ref="N11">EXP(INTERCEPT(LN(E11:H11), LN({7,30,60,90})))</f>
         <v>7.0074738731960559E-2</v>
       </c>
@@ -3057,7 +2543,7 @@
         <f t="shared" si="2"/>
         <v>2.8414942685616955</v>
       </c>
-      <c r="Q11" s="3">
+      <c r="Q11" s="18">
         <f t="shared" si="3"/>
         <v>449.90250720317772</v>
       </c>
@@ -3072,10 +2558,10 @@
     </row>
     <row r="12" spans="1:19">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="B12" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="C12">
         <v>3134</v>
@@ -3099,17 +2585,17 @@
         <v>0.3</v>
       </c>
       <c r="J12" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="L12" t="str">
         <f t="shared" si="0"/>
         <v>applovin_launchpad</v>
       </c>
-      <c r="M12" cm="1">
+      <c r="M12">
         <f t="array" ref="M12">SLOPE(LN(E12:H12), LN({7,30,60,90}))</f>
         <v>0.59287058326121789</v>
       </c>
-      <c r="N12" cm="1">
+      <c r="N12">
         <f t="array" ref="N12">EXP(INTERCEPT(LN(E12:H12), LN({7,30,60,90})))</f>
         <v>3.7251070198513897E-2</v>
       </c>
@@ -3121,7 +2607,7 @@
         <f t="shared" si="2"/>
         <v>1.2309681588606396</v>
       </c>
-      <c r="Q12" s="3">
+      <c r="Q12" s="18">
         <f t="shared" si="3"/>
         <v>705.89068398840459</v>
       </c>
@@ -3136,10 +2622,10 @@
     </row>
     <row r="13" spans="1:19">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="C13">
         <v>1363</v>
@@ -3163,17 +2649,17 @@
         <v>0.22</v>
       </c>
       <c r="J13" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="L13" t="str">
         <f t="shared" si="0"/>
         <v>applovin_wallcraft</v>
       </c>
-      <c r="M13" cm="1">
+      <c r="M13">
         <f t="array" ref="M13">SLOPE(LN(E13:H13), LN({7,30,60,90}))</f>
         <v>0.47201769243271019</v>
       </c>
-      <c r="N13" cm="1">
+      <c r="N13">
         <f t="array" ref="N13">EXP(INTERCEPT(LN(E13:H13), LN({7,30,60,90})))</f>
         <v>4.7413239855488044E-2</v>
       </c>
@@ -3185,7 +2671,7 @@
         <f t="shared" si="2"/>
         <v>0.76797520384903717</v>
       </c>
-      <c r="Q13" s="3">
+      <c r="Q13" s="18">
         <f t="shared" si="3"/>
         <v>2244.4036168319763</v>
       </c>
@@ -3200,10 +2686,10 @@
     </row>
     <row r="14" spans="1:19">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="C14">
         <v>2597</v>
@@ -3227,17 +2713,17 @@
         <v>0.22</v>
       </c>
       <c r="J14" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="L14" t="str">
         <f t="shared" si="0"/>
         <v>tiktok_pingme</v>
       </c>
-      <c r="M14" cm="1">
+      <c r="M14">
         <f t="array" ref="M14">SLOPE(LN(E14:H14), LN({7,30,60,90}))</f>
         <v>0.72041384100071515</v>
       </c>
-      <c r="N14" cm="1">
+      <c r="N14">
         <f t="array" ref="N14">EXP(INTERCEPT(LN(E14:H14), LN({7,30,60,90})))</f>
         <v>1.724117664323311E-2</v>
       </c>
@@ -3249,7 +2735,7 @@
         <f t="shared" si="2"/>
         <v>1.2091443354849851</v>
       </c>
-      <c r="Q14" s="3">
+      <c r="Q14" s="18">
         <f t="shared" si="3"/>
         <v>749.26972565236929</v>
       </c>
@@ -3264,10 +2750,10 @@
     </row>
     <row r="15" spans="1:19">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="B15" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="C15">
         <v>1011</v>
@@ -3291,17 +2777,17 @@
         <v>0.22</v>
       </c>
       <c r="J15" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="L15" t="str">
         <f t="shared" si="0"/>
         <v>applovin_pingme</v>
       </c>
-      <c r="M15" cm="1">
+      <c r="M15">
         <f t="array" ref="M15">SLOPE(LN(E15:H15), LN({7,30,60,90}))</f>
         <v>0.74461976418991838</v>
       </c>
-      <c r="N15" cm="1">
+      <c r="N15">
         <f t="array" ref="N15">EXP(INTERCEPT(LN(E15:H15), LN({7,30,60,90})))</f>
         <v>1.415973462687627E-2</v>
       </c>
@@ -3313,7 +2799,7 @@
         <f t="shared" si="2"/>
         <v>1.1454839875407521</v>
       </c>
-      <c r="Q15" s="3">
+      <c r="Q15" s="18">
         <f t="shared" si="3"/>
         <v>664.73093422199565</v>
       </c>
@@ -3328,10 +2814,10 @@
     </row>
     <row r="16" spans="1:19">
       <c r="A16" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="B16" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="C16">
         <v>2072</v>
@@ -3355,17 +2841,17 @@
         <v>0.2</v>
       </c>
       <c r="J16" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="L16" t="str">
         <f t="shared" si="0"/>
         <v>google_pingme</v>
       </c>
-      <c r="M16" cm="1">
+      <c r="M16">
         <f t="array" ref="M16">SLOPE(LN(E16:H16), LN({7,30,60,90}))</f>
         <v>0.72207165951615448</v>
       </c>
-      <c r="N16" cm="1">
+      <c r="N16">
         <f t="array" ref="N16">EXP(INTERCEPT(LN(E16:H16), LN({7,30,60,90})))</f>
         <v>2.6596801681322096E-2</v>
       </c>
@@ -3377,7 +2863,7 @@
         <f t="shared" si="2"/>
         <v>1.8835991066485438</v>
       </c>
-      <c r="Q16" s="3">
+      <c r="Q16" s="18">
         <f t="shared" si="3"/>
         <v>867.69954894135617</v>
       </c>
@@ -3392,10 +2878,10 @@
     </row>
     <row r="17" spans="1:19">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="B17" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="C17">
         <v>3117</v>
@@ -3419,17 +2905,17 @@
         <v>0.18</v>
       </c>
       <c r="J17" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="L17" t="str">
         <f t="shared" si="0"/>
         <v>meta_pingme</v>
       </c>
-      <c r="M17" cm="1">
+      <c r="M17">
         <f t="array" ref="M17">SLOPE(LN(E17:H17), LN({7,30,60,90}))</f>
         <v>0.68608095016408066</v>
       </c>
-      <c r="N17" cm="1">
+      <c r="N17">
         <f t="array" ref="N17">EXP(INTERCEPT(LN(E17:H17), LN({7,30,60,90})))</f>
         <v>2.5970408443158333E-2</v>
       </c>
@@ -3441,7 +2927,7 @@
         <f t="shared" si="2"/>
         <v>1.4873702924528462</v>
       </c>
-      <c r="Q17" s="3">
+      <c r="Q17" s="18">
         <f t="shared" si="3"/>
         <v>1140.460728670274</v>
       </c>
@@ -3456,37 +2942,38 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>21</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="C2">
         <v>4942.41</v>
@@ -3500,10 +2987,10 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="C3">
         <v>11464.01</v>
@@ -3517,10 +3004,10 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="C4">
         <v>3632.3799999999969</v>
@@ -3534,10 +3021,10 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="C5">
         <v>4975.9599999999973</v>
@@ -3551,10 +3038,10 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="C6">
         <v>19690.48</v>
@@ -3568,10 +3055,10 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="C7">
         <v>44147.740000000013</v>
@@ -3585,10 +3072,10 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="C8">
         <v>14621.33</v>
@@ -3602,10 +3089,10 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="C9">
         <v>19590.28</v>
@@ -3619,10 +3106,10 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="C10">
         <v>26861.89</v>
@@ -3636,10 +3123,10 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="C11">
         <v>60167.87</v>
@@ -3653,10 +3140,10 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="C12">
         <v>20318.139999999981</v>
@@ -3670,10 +3157,10 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="C13">
         <v>27146.11</v>
@@ -3687,10 +3174,10 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="B14" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="C14">
         <v>14609.21</v>
@@ -3704,10 +3191,10 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="B15" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="C15">
         <v>32501.590000000011</v>
@@ -3721,10 +3208,10 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="B16" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="C16">
         <v>10621.53</v>
@@ -3738,10 +3225,10 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="B17" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="C17">
         <v>14840.62</v>
@@ -3759,36 +3246,36 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>23</v>
+        <v>61</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>25</v>
+        <v>63</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>26</v>
+        <v>64</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>27</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="B2">
         <v>305540</v>
@@ -3811,7 +3298,7 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="B3">
         <v>694409</v>
@@ -3834,7 +3321,7 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="B4">
         <v>304868</v>
@@ -3857,7 +3344,7 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="B5">
         <v>228288</v>

</xml_diff>